<commit_message>
progress: 68 village workbooks (sivaramans-llin 2026-10-10T19:10:00Z)
</commit_message>
<xml_diff>
--- a/out/Village_map_of_Tiruvallur_Gummidipoondi_Mangavaram_13.443781_80.155837.xlsx
+++ b/out/Village_map_of_Tiruvallur_Gummidipoondi_Mangavaram_13.443781_80.155837.xlsx
@@ -458,6 +458,11 @@
           <t>100</t>
         </is>
       </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>10, 11A1, 11A2, 11B1, 11B2, 11C1, 11C2, 12A, 12B, 13, 14A, 14B, 15, 16, 17, 1A, 1B1, 1B2, 1B3, 1C, 2, 3, 4, 5, 6, 7, 8A, 8B, 9</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -465,6 +470,11 @@
           <t>101</t>
         </is>
       </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -472,6 +482,11 @@
           <t>102</t>
         </is>
       </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -479,6 +494,11 @@
           <t>103</t>
         </is>
       </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B, 3A1, 3A2, 3B, 4, 5A, 5B</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -486,6 +506,11 @@
           <t>104</t>
         </is>
       </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B, 4A, 4B1, 4B2, 4B3, 5A, 5B, 6</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -493,6 +518,11 @@
           <t>105</t>
         </is>
       </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>10A, 10B, 11A1, 11A2, 11A3, 11B1, 11B2, 11B3A, 11B3B, 12A, 12B, 12C1, 12C2, 1A, 1B, 2A, 2B, 3, 4, 5, 6A, 6B, 6C, 7, 8A, 8B, 8C1, 8C2, 8C3, 8C4, 9A, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -500,6 +530,11 @@
           <t>106</t>
         </is>
       </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -507,6 +542,11 @@
           <t>108</t>
         </is>
       </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -514,6 +554,11 @@
           <t>109</t>
         </is>
       </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6, 7A, 7B, 8</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -521,6 +566,11 @@
           <t>11</t>
         </is>
       </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -528,6 +578,11 @@
           <t>110</t>
         </is>
       </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -535,6 +590,11 @@
           <t>111</t>
         </is>
       </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B1, 3B2</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -542,6 +602,11 @@
           <t>112</t>
         </is>
       </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -549,6 +614,11 @@
           <t>113</t>
         </is>
       </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -556,6 +626,11 @@
           <t>114</t>
         </is>
       </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B, 3A, 3B, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -563,6 +638,11 @@
           <t>115</t>
         </is>
       </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3, 4, 5, 6, 7</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -570,6 +650,11 @@
           <t>116</t>
         </is>
       </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -577,6 +662,11 @@
           <t>117</t>
         </is>
       </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -584,6 +674,11 @@
           <t>118</t>
         </is>
       </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B, 4</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -591,6 +686,11 @@
           <t>119</t>
         </is>
       </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -598,6 +698,11 @@
           <t>12</t>
         </is>
       </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4A, 4B</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -605,6 +710,11 @@
           <t>120</t>
         </is>
       </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -612,6 +722,11 @@
           <t>121</t>
         </is>
       </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -619,6 +734,11 @@
           <t>122</t>
         </is>
       </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -626,6 +746,11 @@
           <t>123</t>
         </is>
       </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>10, 11A, 11B, 12, 13A, 13B, 13C, 13D1, 13D2, 13D3, 13D4, 13E, 14A, 14B, 15, 16A, 16B, 16C, 17, 18, 19A, 19B, 19C, 1A1, 1A2, 2, 3, 4A, 4B, 5, 6, 7, 8, 9A, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -633,6 +758,11 @@
           <t>124</t>
         </is>
       </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 1E, 1F, 1G1, 1G2, 1G3, 1G4, 2A, 2B, 2C, 2D, 2E, 2F, 3A, 3B1, 3B2, 3B3, 3C1, 3C2, 3C3, 4A, 4B, 4C</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -640,6 +770,11 @@
           <t>125</t>
         </is>
       </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -647,6 +782,11 @@
           <t>126</t>
         </is>
       </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -654,6 +794,11 @@
           <t>127</t>
         </is>
       </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B, 3, 4A, 4B, 5A, 5B, 6A, 6B, 6C, 7, 8A, 8B, 9A1A, 9A1B, 9A2, 9A3, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -661,6 +806,11 @@
           <t>128</t>
         </is>
       </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B, 2A, 2B, 2C, 2D, 2E, 3, 4, 5, 6, 7A1, 7A2, 7B, 7C, 7D</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -668,6 +818,11 @@
           <t>129</t>
         </is>
       </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3A1, 3A2, 3B</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -675,6 +830,11 @@
           <t>13</t>
         </is>
       </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A1, 2A2, 2B, 2C, 3, 4A1, 4A2A, 4A2B, 4B, 5A, 5B, 6</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -682,6 +842,11 @@
           <t>130</t>
         </is>
       </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B, 2C, 3, 4A, 4B, 5A, 5B, 6</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -689,6 +854,11 @@
           <t>131</t>
         </is>
       </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>1A, 1B1, 1B2A, 1B2B, 2A, 2B, 3A, 3B</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -696,6 +866,11 @@
           <t>132</t>
         </is>
       </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3A, 3B, 4</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -703,6 +878,11 @@
           <t>133</t>
         </is>
       </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -710,6 +890,11 @@
           <t>134</t>
         </is>
       </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -717,6 +902,11 @@
           <t>135</t>
         </is>
       </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>1A1A1, 1A2, 1B, 2, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -724,6 +914,11 @@
           <t>136</t>
         </is>
       </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -731,6 +926,11 @@
           <t>137</t>
         </is>
       </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B, 3, 4, 5A, 5B, 6</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -738,6 +938,11 @@
           <t>138</t>
         </is>
       </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -745,6 +950,11 @@
           <t>139</t>
         </is>
       </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B, 2A, 2B, 3</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -752,6 +962,11 @@
           <t>14</t>
         </is>
       </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -759,6 +974,11 @@
           <t>140</t>
         </is>
       </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>1A, 1B1A, 1B1B, 1B2, 1B3A, 1B3B, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -766,6 +986,11 @@
           <t>141</t>
         </is>
       </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -773,6 +998,11 @@
           <t>142</t>
         </is>
       </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1A3, 1B1, 1B2, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -780,6 +1010,11 @@
           <t>143</t>
         </is>
       </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C3A1, 1C3B, 1C3C, 2</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -787,6 +1022,11 @@
           <t>144</t>
         </is>
       </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>1A1A, 1B, 1G, 1H, 1I, 2, 3A1, 3A2, 4</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -794,6 +1034,11 @@
           <t>145</t>
         </is>
       </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B1, 2B2</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -801,6 +1046,11 @@
           <t>146</t>
         </is>
       </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -808,6 +1058,11 @@
           <t>147</t>
         </is>
       </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -815,6 +1070,11 @@
           <t>148</t>
         </is>
       </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -822,6 +1082,11 @@
           <t>149</t>
         </is>
       </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -829,6 +1094,11 @@
           <t>15</t>
         </is>
       </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 2A, 2B, 3</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -836,6 +1106,11 @@
           <t>150</t>
         </is>
       </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1A3, 1B, 1C1, 1C2A, 1C2B, 1C2C, 1C2D, 1C2E, 2, 3A, 3B, 4A, 4B</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -843,6 +1118,11 @@
           <t>151</t>
         </is>
       </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 13, 14, 1A, 1B, 2, 3A, 3B1, 3B2, 4A, 4B, 4C, 5, 6, 7, 8A, 8B1A, 8B2, 9</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -850,6 +1130,11 @@
           <t>152</t>
         </is>
       </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>1, 2A1, 2A2, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -857,6 +1142,11 @@
           <t>153</t>
         </is>
       </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -864,6 +1154,11 @@
           <t>154</t>
         </is>
       </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -871,6 +1166,11 @@
           <t>155</t>
         </is>
       </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -878,6 +1178,11 @@
           <t>156</t>
         </is>
       </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4A, 4B</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -885,6 +1190,11 @@
           <t>157</t>
         </is>
       </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -892,6 +1202,11 @@
           <t>158</t>
         </is>
       </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -899,6 +1214,11 @@
           <t>159</t>
         </is>
       </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -906,6 +1226,11 @@
           <t>16</t>
         </is>
       </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3A, 3B</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -913,6 +1238,11 @@
           <t>160</t>
         </is>
       </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -920,6 +1250,11 @@
           <t>161</t>
         </is>
       </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -927,6 +1262,11 @@
           <t>162</t>
         </is>
       </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4A, 4B, 4C, 5</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -934,6 +1274,11 @@
           <t>163</t>
         </is>
       </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -941,6 +1286,11 @@
           <t>164</t>
         </is>
       </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C, 2D, 2E, 3, 4A, 4B, 5</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -948,6 +1298,11 @@
           <t>165</t>
         </is>
       </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3A, 3B, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -955,6 +1310,11 @@
           <t>166</t>
         </is>
       </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -962,6 +1322,11 @@
           <t>167</t>
         </is>
       </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -969,6 +1334,11 @@
           <t>168</t>
         </is>
       </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B, 3C, 4, 5A1, 5A2, 5B, 5C</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -976,6 +1346,11 @@
           <t>169</t>
         </is>
       </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6A, 6B, 7, 8A, 8B, 9A, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -983,6 +1358,11 @@
           <t>17</t>
         </is>
       </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -990,6 +1370,11 @@
           <t>170</t>
         </is>
       </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5A, 5B, 5C, 6A1, 6A2A, 6A2B, 6B1A, 6B1B, 6B2, 6B3, 6B4</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -997,6 +1382,11 @@
           <t>171</t>
         </is>
       </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -1004,6 +1394,11 @@
           <t>172</t>
         </is>
       </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B1, 1B2, 1B3, 2A, 2B, 2C, 3A, 3B, 3C1, 3C2, 4A, 4B</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -1011,6 +1406,11 @@
           <t>173</t>
         </is>
       </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C, 3, 4, 5, 6A, 6B, 7, 8</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -1018,6 +1418,11 @@
           <t>174</t>
         </is>
       </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -1025,6 +1430,11 @@
           <t>175</t>
         </is>
       </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1A3A1A, 1A3A2, 1A3B, 1B, 2A, 2B, 3</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -1032,6 +1442,11 @@
           <t>176</t>
         </is>
       </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>1, 2A1, 2A2, 2B1, 2B2, 2B3, 2C1, 2C2, 2C3</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -1039,6 +1454,11 @@
           <t>177</t>
         </is>
       </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 2A1, 2A2, 2A3, 2B1, 2B2, 2B3, 2B4, 3</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -1046,6 +1466,11 @@
           <t>178</t>
         </is>
       </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -1053,11 +1478,21 @@
           <t>179</t>
         </is>
       </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>10A, 10B, 11, 12, 13A1, 13A2, 13B, 14, 1A, 1B, 1C, 1D, 1E, 2, 3A, 3B1, 3B2, 4A, 4B, 5A, 5B, 5C, 6A, 6B, 7A, 7B, 7C, 8A, 8B, 9A, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
           <t>18</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 2, 3A, 3B, 3C, 4A1, 4A2, 4A3, 4B, 5A, 5B, 6, 7, 8, 9A, 9B</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
progress: 68 village workbooks (sivaramans-llin 2026-10-10T19:20:00Z)
</commit_message>
<xml_diff>
--- a/out/Village_map_of_Tiruvallur_Gummidipoondi_Mangavaram_13.443781_80.155837.xlsx
+++ b/out/Village_map_of_Tiruvallur_Gummidipoondi_Mangavaram_13.443781_80.155837.xlsx
@@ -1502,6 +1502,11 @@
           <t>180</t>
         </is>
       </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B, 1C, 2A1, 2A2, 2A3, 2B, 3</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -1509,6 +1514,11 @@
           <t>181</t>
         </is>
       </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -1516,6 +1526,11 @@
           <t>182</t>
         </is>
       </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 1E, 1F, 2</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -1523,6 +1538,11 @@
           <t>183</t>
         </is>
       </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -1530,6 +1550,11 @@
           <t>184</t>
         </is>
       </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 1A, 1B, 2, 3, 4A, 4B, 5A, 5B, 5C, 6A, 6B, 6C, 7A1, 7A2, 7B1, 7B2, 8A, 8B, 9</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -1537,6 +1562,11 @@
           <t>185</t>
         </is>
       </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -1544,6 +1574,11 @@
           <t>186</t>
         </is>
       </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -1551,6 +1586,11 @@
           <t>187</t>
         </is>
       </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>1, 10A, 10B, 11, 2, 3A, 3B, 3C, 4A, 4B, 5, 6, 7A, 7B, 8, 9A, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -1558,6 +1598,11 @@
           <t>188</t>
         </is>
       </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 2, 3A, 3B, 4A, 4B, 5, 6A, 6B, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -1565,6 +1610,11 @@
           <t>189</t>
         </is>
       </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -1572,6 +1622,11 @@
           <t>19</t>
         </is>
       </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>1, 2A1, 2A2, 2B, 3</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -1579,6 +1634,11 @@
           <t>190</t>
         </is>
       </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -1586,6 +1646,11 @@
           <t>191</t>
         </is>
       </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B1, 1B2, 2A, 2B1, 2B2, 3A1A, 3B, 3C, 3D, 3E</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -1593,6 +1658,11 @@
           <t>192</t>
         </is>
       </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B, 3A, 3B, 4A, 4B, 5A, 5B, 6, 7A, 7B, 8A, 8B, 8C, 9A, 9B1, 9B2, 9C1, 9C2, 9C3, 9D, 9E, 9F, 9G, 9H, 9I1, 9I2, 9I3, 9J, 9K</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -1600,6 +1670,11 @@
           <t>193</t>
         </is>
       </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B, 2A, 2B, 3A, 3B</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -1607,6 +1682,11 @@
           <t>194</t>
         </is>
       </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C1, 1C2, 1D, 1E, 1F, 2A, 2B1, 2B2</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -1614,6 +1694,11 @@
           <t>195</t>
         </is>
       </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B, 4, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -1621,6 +1706,11 @@
           <t>196</t>
         </is>
       </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 2A, 2B, 2C, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -1628,6 +1718,11 @@
           <t>197</t>
         </is>
       </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C, 3A, 3B, 3C, 3D, 4A, 4B, 4C, 5A, 5B, 5C</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -1635,6 +1730,11 @@
           <t>198</t>
         </is>
       </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -1642,6 +1742,11 @@
           <t>199</t>
         </is>
       </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -1649,6 +1754,11 @@
           <t>2</t>
         </is>
       </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6, 7, 8</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -1656,6 +1766,11 @@
           <t>20</t>
         </is>
       </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3, 4A, 4B, 4C, 4D</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -1663,6 +1778,11 @@
           <t>200</t>
         </is>
       </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 2, 3, 4A, 4B, 5, 6, 7A1A, 7A1B, 7A1C, 7A2, 7A3, 7B, 8, 9A, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -1670,6 +1790,11 @@
           <t>201</t>
         </is>
       </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -1677,6 +1802,11 @@
           <t>202</t>
         </is>
       </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>1A, 1B1, 1B2, 2A, 2B1, 2B2A, 2B2B</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -1684,6 +1814,11 @@
           <t>203</t>
         </is>
       </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>1, 10A, 10B, 2A, 2B, 3A1, 3A2, 3B, 4A1, 4A2, 4B1, 4B2, 5A, 5B, 6, 7, 8A, 8B, 9A, 9B, 9C</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -1691,6 +1826,11 @@
           <t>204</t>
         </is>
       </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B1, 3B2, 4</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -1698,6 +1838,11 @@
           <t>205</t>
         </is>
       </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -1705,6 +1850,11 @@
           <t>206</t>
         </is>
       </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B1A, 2B1B, 2B2</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -1712,6 +1862,11 @@
           <t>207</t>
         </is>
       </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>1, 2A1, 2A2, 2B, 3, 4, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -1719,6 +1874,11 @@
           <t>208</t>
         </is>
       </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>1, 2A1, 2A2, 2B, 3, 4A, 4B, 5A1, 5A2, 5B, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -1726,6 +1886,11 @@
           <t>209</t>
         </is>
       </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B, 2A, 2B, 3A, 3B, 4A, 4B, 5</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -1733,6 +1898,11 @@
           <t>21</t>
         </is>
       </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B, 1C1, 1C2, 2</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -1740,6 +1910,11 @@
           <t>210</t>
         </is>
       </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C1, 1C2, 1C3, 2</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -1747,6 +1922,11 @@
           <t>211</t>
         </is>
       </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12A1, 12A2, 12B, 2A, 2B, 3, 4A, 4B, 5A, 5B, 6A1, 6A2, 6B, 6C, 6D1, 6D2, 7A1, 7A2, 7B1, 7B2A, 7B2B, 8A, 8B, 9</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -1754,6 +1934,11 @@
           <t>212</t>
         </is>
       </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -1761,6 +1946,11 @@
           <t>213</t>
         </is>
       </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>1, 2A1, 2A2, 2B, 2C1, 2C2, 3A, 3B, 4A, 4B, 5, 6, 7</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -1768,6 +1958,11 @@
           <t>214</t>
         </is>
       </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 1E1, 1E2, 2A1, 2A2, 2B1, 2B2</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -1775,6 +1970,11 @@
           <t>215</t>
         </is>
       </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B, 3, 4, 5A, 5B</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -1782,6 +1982,11 @@
           <t>216</t>
         </is>
       </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B1, 2B2, 2B3, 2C1, 2C2</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -1789,6 +1994,11 @@
           <t>217</t>
         </is>
       </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>1A, 1B1, 1B2, 1C, 1D, 1E1, 1E2, 1F1, 1F2, 1G, 1H1, 1H2, 1J1, 1J2, 1K, 1L, 2A, 2B, 9I</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -1796,6 +2006,11 @@
           <t>218</t>
         </is>
       </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B, 4A, 4B</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -1803,6 +2018,11 @@
           <t>219</t>
         </is>
       </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 13A, 13B, 1A, 1B, 1C, 2A, 2B, 3A, 3B, 4A1, 4A2, 4B1, 4B2, 5, 6A, 6B, 7, 8A, 8B, 8C, 9A, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -1810,6 +2030,11 @@
           <t>22</t>
         </is>
       </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -1817,6 +2042,11 @@
           <t>220</t>
         </is>
       </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 2A, 2B, 2C, 2D, 2E, 3A, 3B, 3C</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -1824,6 +2054,11 @@
           <t>221</t>
         </is>
       </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -1831,6 +2066,11 @@
           <t>222</t>
         </is>
       </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -1838,6 +2078,11 @@
           <t>223</t>
         </is>
       </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -1845,6 +2090,11 @@
           <t>224</t>
         </is>
       </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>1, 2, 3A1, 3A2, 3B, 3C1, 3C2A1, 3C2B, 4, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -1852,6 +2102,11 @@
           <t>225</t>
         </is>
       </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>1, 2A1A, 2A1B, 2A2, 2A3, 2B, 3A1, 3A2, 3A3, 3B, 3C1, 3C2, 4A, 4B, 4C, 4D</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -1859,6 +2114,11 @@
           <t>226</t>
         </is>
       </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -1866,6 +2126,11 @@
           <t>227</t>
         </is>
       </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -1873,6 +2138,11 @@
           <t>228</t>
         </is>
       </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>1A1A, 1A1B, 1A2, 1B, 1C, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -1880,6 +2150,11 @@
           <t>229</t>
         </is>
       </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -1887,6 +2162,11 @@
           <t>23</t>
         </is>
       </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C, 2D, 3</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -1894,6 +2174,11 @@
           <t>230</t>
         </is>
       </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -1901,6 +2186,11 @@
           <t>231</t>
         </is>
       </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -1908,6 +2198,11 @@
           <t>232</t>
         </is>
       </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B1, 1B2, 1C1, 1C2, 2</t>
+        </is>
+      </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -1915,6 +2210,11 @@
           <t>233</t>
         </is>
       </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -1922,6 +2222,11 @@
           <t>234</t>
         </is>
       </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C1, 1C2, 2</t>
+        </is>
+      </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -1929,6 +2234,11 @@
           <t>235</t>
         </is>
       </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3, 4A, 4B</t>
+        </is>
+      </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
@@ -1936,6 +2246,11 @@
           <t>236</t>
         </is>
       </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A1, 2A2, 2A3, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
@@ -1943,6 +2258,11 @@
           <t>237</t>
         </is>
       </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 1A, 1B, 20, 21, 22, 23, 24, 25, 2A1A1A, 2A1B1, 2A1C1, 2A2, 2B, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -1950,6 +2270,11 @@
           <t>238</t>
         </is>
       </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
@@ -1957,6 +2282,11 @@
           <t>239</t>
         </is>
       </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 13, 14, 15, 16, 1A1A, 1A1B, 1A1C, 1A2, 1A3, 1A4, 1B1, 1B2, 2A1, 2B, 2C, 2D, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
@@ -1964,6 +2294,11 @@
           <t>24</t>
         </is>
       </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3A, 3B1, 3B2</t>
+        </is>
+      </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
@@ -1971,6 +2306,11 @@
           <t>240</t>
         </is>
       </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
@@ -1978,6 +2318,11 @@
           <t>241</t>
         </is>
       </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
@@ -1985,6 +2330,11 @@
           <t>242</t>
         </is>
       </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>1A, 1A2A, 1A2B, 1A2C, 1A2D1A, 1A2D1B, 1A2D2, 1A3A1, 1A3A2, 1A3A3A, 1A3B1, 1B, 2A, 2B1, 2B2, 2B3, 2B4, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
@@ -1992,6 +2342,11 @@
           <t>243</t>
         </is>
       </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
@@ -1999,6 +2354,11 @@
           <t>244</t>
         </is>
       </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
@@ -2006,6 +2366,11 @@
           <t>245</t>
         </is>
       </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
@@ -2013,11 +2378,21 @@
           <t>246</t>
         </is>
       </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6, 7</t>
+        </is>
+      </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
           <t>247</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B1, 1B2, 2A, 2B, 2C</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
progress: 68 village workbooks (sivaramans-llin 2026-10-10T19:30:00Z)
</commit_message>
<xml_diff>
--- a/out/Village_map_of_Tiruvallur_Gummidipoondi_Mangavaram_13.443781_80.155837.xlsx
+++ b/out/Village_map_of_Tiruvallur_Gummidipoondi_Mangavaram_13.443781_80.155837.xlsx
@@ -2402,6 +2402,11 @@
           <t>248</t>
         </is>
       </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
@@ -2409,6 +2414,11 @@
           <t>249</t>
         </is>
       </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 1E, 2, 3, 4A, 4B, 4C, 4D</t>
+        </is>
+      </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
@@ -2416,6 +2426,11 @@
           <t>25</t>
         </is>
       </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>1A1A, 1A1B, 1A2A, 1A2B, 1B1A, 1B1B, 1B2A, 1B2B, 1B3, 2</t>
+        </is>
+      </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
@@ -2423,6 +2438,11 @@
           <t>250</t>
         </is>
       </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B, 1C, 2, 3A, 3B1, 3B2, 3B3</t>
+        </is>
+      </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
@@ -2430,6 +2450,11 @@
           <t>251</t>
         </is>
       </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
@@ -2437,6 +2462,11 @@
           <t>252</t>
         </is>
       </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
@@ -2444,6 +2474,11 @@
           <t>253</t>
         </is>
       </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>1A, 1B1A, 1B1B, 1B2A1, 1B2B, 1B2C, 1B2D, 1C, 1D, 1E, 1F, 1G1, 1G2, 2, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
@@ -2451,6 +2486,11 @@
           <t>254</t>
         </is>
       </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 2</t>
+        </is>
+      </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
@@ -2458,6 +2498,11 @@
           <t>255</t>
         </is>
       </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
@@ -2465,6 +2510,11 @@
           <t>256</t>
         </is>
       </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5A, 5B, 6, 7A1, 7A10, 7A11, 7A2, 7A3, 7A4, 7A5, 7A6, 7A7, 7A8, 7A9, 7B</t>
+        </is>
+      </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
@@ -2472,6 +2522,11 @@
           <t>257</t>
         </is>
       </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>1A1, 1A10, 1A11, 1A12, 1A13, 1A14, 1A15, 1A16, 1A17, 1A18, 1A19, 1A2, 1A20, 1A21, 1A22, 1A23, 1A24, 1A25, 1A3, 1A4A, 1A4B, 1A5, 1A6, 1A7, 1A8, 1A9</t>
+        </is>
+      </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
@@ -2479,6 +2534,11 @@
           <t>258</t>
         </is>
       </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>10A, 10B, 11, 1A1, 1A2, 1B, 1C, 2, 3A1, 3A2, 3B, 3C, 3D, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
@@ -2486,6 +2546,11 @@
           <t>259</t>
         </is>
       </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
@@ -2493,6 +2558,11 @@
           <t>26</t>
         </is>
       </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B, 4, 5, 6, 7</t>
+        </is>
+      </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
@@ -2500,6 +2570,11 @@
           <t>260</t>
         </is>
       </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B, 3A1, 3A2, 3B, 4</t>
+        </is>
+      </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
@@ -2507,6 +2582,11 @@
           <t>261</t>
         </is>
       </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
@@ -2514,6 +2594,11 @@
           <t>262</t>
         </is>
       </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B, 2A1, 2A2, 2B, 3A, 3B, 4A, 4B1, 4B2</t>
+        </is>
+      </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
@@ -2521,6 +2606,11 @@
           <t>263</t>
         </is>
       </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3A, 3B, 4A, 4B, 4C1, 4C2, 4C3</t>
+        </is>
+      </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
@@ -2528,6 +2618,11 @@
           <t>264</t>
         </is>
       </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
@@ -2535,6 +2630,11 @@
           <t>265</t>
         </is>
       </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B1A, 1B1B, 1B2A, 1B2B1, 1B2B2A1, 2A1A, 2A1B, 2A2, 2A3, 2A4, 2A5, 2A6, 2A7, 2B, 2C, 2D, 3, 4, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
@@ -2542,6 +2642,11 @@
           <t>266</t>
         </is>
       </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
@@ -2549,6 +2654,11 @@
           <t>267</t>
         </is>
       </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
@@ -2556,6 +2666,11 @@
           <t>268</t>
         </is>
       </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>1A1A1, 1A1B, 1A2A, 1A2B, 1A3A1, 1B, 1C, 2, 3, 4, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
@@ -2563,6 +2678,11 @@
           <t>269</t>
         </is>
       </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>10, 1A, 1B, 1C, 1D, 2A, 2B, 2C1, 2C2, 2C3, 2D1, 2D2, 3A1A, 3A1B1, 3A1B2, 3A2A, 3A3A1, 3A3B, 3B, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
@@ -2570,6 +2690,11 @@
           <t>27</t>
         </is>
       </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3, 4, 5, 6A, 6B</t>
+        </is>
+      </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
@@ -2577,6 +2702,11 @@
           <t>270</t>
         </is>
       </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B, 2A1, 2A2, 2B, 2C, 3A1, 3A2, 3B, 3C, 3D, 4A, 4B, 4C, 5A, 5B1, 5B2, 5B3, 5B4, 5C, 5D, 5E, 5F1, 5F2, 5F3, 6A1, 6A2, 6A3, 6A4, 6B, 6C1A, 6C1B, 6C2, 7A1, 7A2, 7B1, 7B2, 7B3, 7C1, 7C2, 7C3, 8A1, 8A2, 8A3, 8B1, 8B2, 8B3, 8C1, 8C2, 8C3</t>
+        </is>
+      </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
@@ -2584,6 +2714,11 @@
           <t>271</t>
         </is>
       </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B1, 1B2, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
@@ -2591,6 +2726,11 @@
           <t>272</t>
         </is>
       </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 2A, 2B, 3A, 3B, 4, 5A, 5B, 5C, 5D, 5E, 6A1A1A, 6A1A2, 6A1A3, 6A1A4A1A, 6A1A5A, 6A1A5B, 6A1A6, 6A1B, 6A2A, 6A2B, 6B1A1A, 6B1B, 6B1C, 6B1D, 6B1E, 6B1F, 6B1G, 6B2, 6C1A1, 6C1A2, 6C1B, 6C1C, 6C2, 6C3, 6C4, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
@@ -2598,6 +2738,11 @@
           <t>273</t>
         </is>
       </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
@@ -2605,6 +2750,11 @@
           <t>274</t>
         </is>
       </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>1, 2A1, 2A2, 2B, 3A, 3B, 3C, 4</t>
+        </is>
+      </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
@@ -2612,6 +2762,11 @@
           <t>275</t>
         </is>
       </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>10, 1A, 1B, 2A, 2B, 3, 4, 5A, 5B, 6, 7, 8A1, 8A2, 8B, 9</t>
+        </is>
+      </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
@@ -2619,6 +2774,11 @@
           <t>276</t>
         </is>
       </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3, 4A, 4B, 4C, 4D</t>
+        </is>
+      </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
@@ -2626,6 +2786,11 @@
           <t>277</t>
         </is>
       </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B, 3</t>
+        </is>
+      </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
@@ -2633,6 +2798,11 @@
           <t>278</t>
         </is>
       </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B, 2A, 2B, 3, 4A, 4B</t>
+        </is>
+      </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
@@ -2640,6 +2810,11 @@
           <t>279</t>
         </is>
       </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>10, 11, 12A1, 12B, 12C, 13A, 13B, 13C, 14A, 14B, 14C, 15A, 15B, 16, 17A, 17B, 17C, 18, 19, 1A1, 1A2, 1A3, 1B, 2, 20, 21A, 21B, 22A, 22B, 22C, 23A, 23B, 24A, 24B, 25A, 25B, 26A, 26B, 27A, 27B, 28A, 28B, 29, 3, 30, 31, 32, 33A, 33B, 34, 4, 5, 6, 7, 8A, 8B, 9</t>
+        </is>
+      </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
@@ -2647,6 +2822,11 @@
           <t>28</t>
         </is>
       </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 1E, 2A, 2B, 2C, 2D, 3A1, 3A2, 3A3, 3B, 3C</t>
+        </is>
+      </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
@@ -2654,6 +2834,11 @@
           <t>280</t>
         </is>
       </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>1, 10, 2, 3, 4A, 4B, 5A, 5B, 6A, 6B, 7A, 7B, 7C, 8A, 8B, 9A, 9B, 9C</t>
+        </is>
+      </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
@@ -2661,6 +2846,11 @@
           <t>281</t>
         </is>
       </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B, 2A, 2B, 3</t>
+        </is>
+      </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
@@ -2668,6 +2858,11 @@
           <t>282</t>
         </is>
       </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
@@ -2675,6 +2870,11 @@
           <t>283</t>
         </is>
       </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
@@ -2682,6 +2882,11 @@
           <t>29</t>
         </is>
       </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A1, 2A2, 2A3, 2B, 3A, 3B, 4A, 4B, 5A, 5B, 6A, 6B</t>
+        </is>
+      </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
@@ -2689,6 +2894,11 @@
           <t>3</t>
         </is>
       </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>1, 2, 3A1, 3A2, 3B, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
@@ -2696,6 +2906,11 @@
           <t>30</t>
         </is>
       </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3A, 3B, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
@@ -2703,6 +2918,11 @@
           <t>31</t>
         </is>
       </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B, 4, 5, 6, 7A, 7B</t>
+        </is>
+      </c>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
@@ -2710,6 +2930,11 @@
           <t>32</t>
         </is>
       </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4A, 4B, 5, 6, 7</t>
+        </is>
+      </c>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
@@ -2717,6 +2942,11 @@
           <t>33</t>
         </is>
       </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
@@ -2724,6 +2954,11 @@
           <t>34</t>
         </is>
       </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1A3, 1B, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
@@ -2731,6 +2966,11 @@
           <t>35</t>
         </is>
       </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
@@ -2738,6 +2978,11 @@
           <t>36</t>
         </is>
       </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
@@ -2745,6 +2990,11 @@
           <t>37</t>
         </is>
       </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
@@ -2752,6 +3002,11 @@
           <t>38</t>
         </is>
       </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
@@ -2759,6 +3014,11 @@
           <t>39</t>
         </is>
       </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B</t>
+        </is>
+      </c>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
@@ -2766,6 +3026,11 @@
           <t>4</t>
         </is>
       </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5A, 5B</t>
+        </is>
+      </c>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
@@ -2773,6 +3038,11 @@
           <t>40</t>
         </is>
       </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>1, 2, 3A1, 3A2, 3B, 4</t>
+        </is>
+      </c>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
@@ -2780,6 +3050,11 @@
           <t>41</t>
         </is>
       </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2</t>
+        </is>
+      </c>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
@@ -2787,6 +3062,11 @@
           <t>42</t>
         </is>
       </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
@@ -2794,6 +3074,11 @@
           <t>43</t>
         </is>
       </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
@@ -2801,6 +3086,11 @@
           <t>44</t>
         </is>
       </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 2</t>
+        </is>
+      </c>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
@@ -2808,6 +3098,11 @@
           <t>45</t>
         </is>
       </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5A, 5B</t>
+        </is>
+      </c>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
@@ -2815,6 +3110,11 @@
           <t>46</t>
         </is>
       </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4A, 4B, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
@@ -2822,6 +3122,11 @@
           <t>47</t>
         </is>
       </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3A, 3B1, 3B2</t>
+        </is>
+      </c>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
@@ -2829,6 +3134,11 @@
           <t>48</t>
         </is>
       </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
@@ -2836,6 +3146,11 @@
           <t>49</t>
         </is>
       </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B, 2C</t>
+        </is>
+      </c>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
@@ -2843,6 +3158,11 @@
           <t>5</t>
         </is>
       </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
@@ -2850,6 +3170,11 @@
           <t>50</t>
         </is>
       </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
@@ -2857,6 +3182,11 @@
           <t>51</t>
         </is>
       </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2</t>
+        </is>
+      </c>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
@@ -2864,6 +3194,11 @@
           <t>52</t>
         </is>
       </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
@@ -2871,6 +3206,11 @@
           <t>53</t>
         </is>
       </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3, 4A, 4B</t>
+        </is>
+      </c>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
@@ -2878,6 +3218,11 @@
           <t>54</t>
         </is>
       </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6, 7</t>
+        </is>
+      </c>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
@@ -2885,6 +3230,11 @@
           <t>55</t>
         </is>
       </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
@@ -2892,6 +3242,11 @@
           <t>56</t>
         </is>
       </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>1, 2A1, 2A2, 2B, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
@@ -2899,6 +3254,11 @@
           <t>57</t>
         </is>
       </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C, 3</t>
+        </is>
+      </c>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
@@ -2906,6 +3266,11 @@
           <t>58</t>
         </is>
       </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C, 3, 4A1, 4A2, 4A3, 4A4, 4B</t>
+        </is>
+      </c>
     </row>
     <row r="239">
       <c r="A239" t="inlineStr">
@@ -2913,6 +3278,11 @@
           <t>59</t>
         </is>
       </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B, 2A, 2B, 2C, 2D1, 2D2, 3A, 3B1, 3B2, 3C</t>
+        </is>
+      </c>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
@@ -2920,6 +3290,11 @@
           <t>6</t>
         </is>
       </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3A, 3B, 4A, 4B, 5, 6, 7</t>
+        </is>
+      </c>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
@@ -2927,6 +3302,11 @@
           <t>60</t>
         </is>
       </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
@@ -2934,6 +3314,11 @@
           <t>61</t>
         </is>
       </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C, 2D</t>
+        </is>
+      </c>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
@@ -2941,6 +3326,11 @@
           <t>62</t>
         </is>
       </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
@@ -2948,6 +3338,11 @@
           <t>63</t>
         </is>
       </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3, 4A, 4B, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
@@ -2955,6 +3350,11 @@
           <t>64</t>
         </is>
       </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
@@ -2962,11 +3362,21 @@
           <t>65</t>
         </is>
       </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4A, 4B1, 4B2, 4C, 5A, 5B, 6, 7A, 7B</t>
+        </is>
+      </c>
     </row>
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
           <t>66</t>
+        </is>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
progress: 69 village workbooks (sivaramans-llin 2026-10-10T19:40:00Z)
</commit_message>
<xml_diff>
--- a/out/Village_map_of_Tiruvallur_Gummidipoondi_Mangavaram_13.443781_80.155837.xlsx
+++ b/out/Village_map_of_Tiruvallur_Gummidipoondi_Mangavaram_13.443781_80.155837.xlsx
@@ -3386,6 +3386,11 @@
           <t>67</t>
         </is>
       </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3</t>
+        </is>
+      </c>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
@@ -3393,6 +3398,11 @@
           <t>68</t>
         </is>
       </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="250">
       <c r="A250" t="inlineStr">
@@ -3400,6 +3410,11 @@
           <t>69</t>
         </is>
       </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="251">
       <c r="A251" t="inlineStr">
@@ -3407,6 +3422,11 @@
           <t>7</t>
         </is>
       </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="252">
       <c r="A252" t="inlineStr">
@@ -3414,6 +3434,11 @@
           <t>70</t>
         </is>
       </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="253">
       <c r="A253" t="inlineStr">
@@ -3421,6 +3446,11 @@
           <t>71</t>
         </is>
       </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="254">
       <c r="A254" t="inlineStr">
@@ -3428,6 +3458,11 @@
           <t>73</t>
         </is>
       </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="255">
       <c r="A255" t="inlineStr">
@@ -3435,6 +3470,11 @@
           <t>74</t>
         </is>
       </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="256">
       <c r="A256" t="inlineStr">
@@ -3442,6 +3482,11 @@
           <t>75</t>
         </is>
       </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4A, 4B, 5, 6A, 6B, 7A, 7B, 8A, 8B</t>
+        </is>
+      </c>
     </row>
     <row r="257">
       <c r="A257" t="inlineStr">
@@ -3449,6 +3494,11 @@
           <t>76</t>
         </is>
       </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2</t>
+        </is>
+      </c>
     </row>
     <row r="258">
       <c r="A258" t="inlineStr">
@@ -3456,6 +3506,11 @@
           <t>77</t>
         </is>
       </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>1, 10A, 10B, 11A, 11B, 12, 2, 3A, 3B, 4A, 4B, 5A, 5B, 6A, 6B, 7A, 7B, 7C, 7D, 8, 9A, 9B, 9C</t>
+        </is>
+      </c>
     </row>
     <row r="259">
       <c r="A259" t="inlineStr">
@@ -3463,6 +3518,11 @@
           <t>78</t>
         </is>
       </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="260">
       <c r="A260" t="inlineStr">
@@ -3470,6 +3530,11 @@
           <t>79</t>
         </is>
       </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="261">
       <c r="A261" t="inlineStr">
@@ -3477,6 +3542,11 @@
           <t>8</t>
         </is>
       </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="262">
       <c r="A262" t="inlineStr">
@@ -3484,6 +3554,11 @@
           <t>80</t>
         </is>
       </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">
@@ -3491,6 +3566,11 @@
           <t>81</t>
         </is>
       </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="264">
       <c r="A264" t="inlineStr">
@@ -3498,6 +3578,11 @@
           <t>82</t>
         </is>
       </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C</t>
+        </is>
+      </c>
     </row>
     <row r="265">
       <c r="A265" t="inlineStr">
@@ -3505,6 +3590,11 @@
           <t>83</t>
         </is>
       </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="266">
       <c r="A266" t="inlineStr">
@@ -3512,6 +3602,11 @@
           <t>84</t>
         </is>
       </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 2, 3A, 3B, 4</t>
+        </is>
+      </c>
     </row>
     <row r="267">
       <c r="A267" t="inlineStr">
@@ -3519,6 +3614,11 @@
           <t>85</t>
         </is>
       </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B1, 1B2, 2A, 2B, 2C1, 2C2</t>
+        </is>
+      </c>
     </row>
     <row r="268">
       <c r="A268" t="inlineStr">
@@ -3526,6 +3626,11 @@
           <t>86</t>
         </is>
       </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 2, 3, 4A, 4B, 5, 6, 7, 8, 9A, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="269">
       <c r="A269" t="inlineStr">
@@ -3533,6 +3638,11 @@
           <t>87</t>
         </is>
       </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2</t>
+        </is>
+      </c>
     </row>
     <row r="270">
       <c r="A270" t="inlineStr">
@@ -3540,6 +3650,11 @@
           <t>88</t>
         </is>
       </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B, 1C, 2</t>
+        </is>
+      </c>
     </row>
     <row r="271">
       <c r="A271" t="inlineStr">
@@ -3547,6 +3662,11 @@
           <t>89</t>
         </is>
       </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="272">
       <c r="A272" t="inlineStr">
@@ -3554,6 +3674,11 @@
           <t>9</t>
         </is>
       </c>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 1E, 1F, 1G, 1H, 1I, 1J, 2A, 2B, 2C, 2D, 2E</t>
+        </is>
+      </c>
     </row>
     <row r="273">
       <c r="A273" t="inlineStr">
@@ -3561,6 +3686,11 @@
           <t>90</t>
         </is>
       </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3, 4A1, 4A2, 4B, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="274">
       <c r="A274" t="inlineStr">
@@ -3568,6 +3698,11 @@
           <t>91</t>
         </is>
       </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>1A1A1, 1A1B, 1A2, 1B, 2, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="275">
       <c r="A275" t="inlineStr">
@@ -3575,6 +3710,11 @@
           <t>92</t>
         </is>
       </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="276">
       <c r="A276" t="inlineStr">
@@ -3582,6 +3722,11 @@
           <t>93</t>
         </is>
       </c>
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="277">
       <c r="A277" t="inlineStr">
@@ -3589,6 +3734,11 @@
           <t>94</t>
         </is>
       </c>
+      <c r="B277" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A1, 2A1A, 2A1B, 2A1C, 2A1D, 2A1E, 2A1F, 2A1G, 2A1H, 2A1J1, 2A1J2, 2A1J3, 2A1K, 2A1L, 2A1M, 2A2, 2A3, 2A4, 2A5, 2A6, 2A7, 2A8, 2A9, 2B1, 2B2, 3A, 3B, 3C</t>
+        </is>
+      </c>
     </row>
     <row r="278">
       <c r="A278" t="inlineStr">
@@ -3596,6 +3746,11 @@
           <t>95</t>
         </is>
       </c>
+      <c r="B278" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="279">
       <c r="A279" t="inlineStr">
@@ -3603,6 +3758,11 @@
           <t>96</t>
         </is>
       </c>
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="280">
       <c r="A280" t="inlineStr">
@@ -3610,6 +3770,11 @@
           <t>97</t>
         </is>
       </c>
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>1, 2A1A, 2A1B, 2A2, 2B, 3, 4A1A, 4A1B, 4A1C, 4A2, 4B, 4C, 4D</t>
+        </is>
+      </c>
     </row>
     <row r="281">
       <c r="A281" t="inlineStr">
@@ -3617,11 +3782,21 @@
           <t>98</t>
         </is>
       </c>
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B, 2, 3, 4, 5, 6, 7A, 7B, 8, 9A1, 9A2A, 9A2B, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="282">
       <c r="A282" t="inlineStr">
         <is>
           <t>99</t>
+        </is>
+      </c>
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4A, 4B1, 4B2</t>
         </is>
       </c>
     </row>

</xml_diff>